<commit_message>
Draw Monguno with the fixed draw script; mark Kala/Balge, Ngala and Nganzai not recoverable by hand
On Jack's direct word. Monguno: 2 full clusters, all 24 households
accessible, merged; 10.55% -> 9.88%, Representative (255 national).
The three Borno strata stay labelled recoverable in 05, whose pool is an
unvalidated hex count, but the building-validated draw shows no draw can
close them; the donor classification now marks them not recoverable with
that evidence, in its own column.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resampling/input/accessibility_reports_returned/Street Child of Nigeria_accessibility_report.xlsx
+++ b/resampling/input/accessibility_reports_returned/Street Child of Nigeria_accessibility_report.xlsx
@@ -223,8 +223,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClusterAccessibility" displayName="ClusterAccessibility" ref="A1:O74" headerRowCount="1">
-  <autoFilter ref="A1:O74"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClusterAccessibility" displayName="ClusterAccessibility" ref="A1:O76" headerRowCount="1">
+  <autoFilter ref="A1:O76"/>
   <tableColumns count="15">
     <tableColumn id="1" name="State"/>
     <tableColumn id="2" name="LGA"/>
@@ -2925,7 +2925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O74"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14" customWidth="1" style="12" min="1" max="2"/>
@@ -5864,7 +5864,6 @@
           <t>non_idp_NG008024_supp31</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>6</t>
@@ -5902,13 +5901,88 @@
           <t>non_idp_NG008024_supp32</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Borno</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Monguno</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Monguno</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Non-IDP</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>non_idp_NG008024_supp33</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Borno</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Monguno</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Monguno</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Non-IDP</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>non_idp_NG008024_supp34</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -5916,19 +5990,19 @@
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation sqref="I2:I74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"N/A - fully accessible,Insecurity / conflict,Physical access (terrain, flooding, roads),Population absent / relocated,Building-footprint issue (no eligible structures),Access denied by authorities / community,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Partner,IMPACT (default - accessible until reported otherwise)"</formula1>
     </dataValidation>
-    <dataValidation sqref="O2:O74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O2:O76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Partner's own template,Email,WhatsApp/verbal (coordinator-transcribed),Point-level file annotation,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date">
+    <dataValidation sqref="M2:M76" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date">
       <formula1>2026-7-1</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>